<commit_message>
Add research reports: COHR, CLS, ARM, NOW, FN; refresh AVGO
Full STUPIDMEI deliverables per ticker (inputs + valuation + narrative JSON,
xlsx, pdf). DCF for COHR/CLS/ARM/NOW/FN, SOTP for AVGO. Valuations produced
by the deterministic compute scripts; narratives voice-cleaned and rendered
via the locked Excel/PDF templates.

Intrinsic-value read: COHR/CLS/ARM/FN screen well above intrinsic after large
AI-driven re-rates (SELL); NOW roughly fair (HOLD); AVGO HOLD with negative bias.

https://claude.ai/code/session_016hSKJbwb3rtsFFuTsbZRja
</commit_message>
<xml_diff>
--- a/output/AVGO/AVGO.xlsx
+++ b/output/AVGO/AVGO.xlsx
@@ -547,7 +547,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Institutional Equity Research  |  Date: 2026-06-09  |  Listings: NASDAQ  |  Engine: himself65/finance-skills</t>
+          <t>Institutional Equity Research  |  Date: 2026-06-10  |  Listings: NASDAQ  |  Engine: himself65/finance-skills</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>$371</t>
+          <t>$368</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>$397</t>
+          <t>$392</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>-6.5%</t>
+          <t>-6.1%</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>$370</t>
+          <t>$368</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>-6.7%</t>
+          <t>-6.1%</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>$396.60</t>
+          <t>$392.16</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>195.86</v>
+        <v>194.93</v>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
       <c r="F5" s="8" t="inlineStr">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>370</v>
+        <v>368.25</v>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
       <c r="F6" s="8" t="inlineStr">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>566.55</v>
+        <v>563.86</v>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D10" s="21" t="n">
-        <v>370</v>
+        <v>368.25</v>
       </c>
     </row>
     <row r="11">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>396.6</v>
+        <v>392.16</v>
       </c>
     </row>
     <row r="12">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D12" s="18" t="n">
-        <v>-0.067</v>
+        <v>-0.061</v>
       </c>
     </row>
     <row r="13"/>

</xml_diff>

<commit_message>
Add formal audits, AVGO reconciliation, and ecosystem+reports explainer
- equity-audit run on all six (COHR, CLS, ARM, NOW, FN, AVGO): PASS_WITH_NOTES,
  every valuation reproduces byte-for-byte. Audit caught and corrected a
  probability-sum error (1.05 -> 1.0) in COHR and FN.
- AVGO target reconciled: narrative now uses the probability-weighted blend
  ($370) while disclosing the base SOTP aggregate ($368).
- New explainer output/SEMICONDUCTOR_ECOSYSTEM_AND_REPORTS.md: the value-chain
  visual map (front/back-end, interconnect, manufacturing/test, assembly,
  photonics, storage) plus the six reports, audit results, and a reverse-DCF
  bridge explaining why intrinsic targets sit below Street (market is paying
  2.5-7.75x our base-case FCF; price is above our Bull case for four of five).

https://claude.ai/code/session_016hSKJbwb3rtsFFuTsbZRja
</commit_message>
<xml_diff>
--- a/output/AVGO/AVGO.xlsx
+++ b/output/AVGO/AVGO.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>$368</t>
+          <t>$370</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>-6.1%</t>
+          <t>-5.8%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AVGO rerun: BUY $450 target (+19.5%), SOTP $477 base, updated Q2-FY26 data
Full rerun incorporating Q2-FY26 8-K data: AI semi $10.8bn (+143% YoY),
Q3-FY26 guide $29.4bn / $16bn AI, FY27 AI guide >$100bn. SOTP method:
Semi DCF ($32B-$105B FCF, WACC 8.25%, g 4.25%) + VMware 17x $22B EBITDA.
Bear $251 / Base $477 / Bull $733. Probability-weighted target $450.
Fixed voice_clean.py em-dash bug (dropped first char after dash).
Fixed render_pdf.py null geo-pct crash. Audit: PASS_WITH_NOTES (WACC
component gap flagged; 52w low corrected to $244.17).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wv887Z52HwZ5Pqm6eYCtA
</commit_message>
<xml_diff>
--- a/output/AVGO/AVGO.xlsx
+++ b/output/AVGO/AVGO.xlsx
@@ -92,12 +92,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -117,7 +112,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,34 +133,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -547,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Institutional Equity Research  |  Date: 2026-06-10  |  Listings: NASDAQ  |  Engine: himself65/finance-skills</t>
+          <t>Institutional Equity Research  |  Date: 2026-06-17  |  Listings: NASDAQ  |  Engine: himself65/finance-skills</t>
         </is>
       </c>
     </row>
@@ -560,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>HOLD with negative bias</t>
+          <t>BUY with positive bias</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -570,7 +571,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>$370</t>
+          <t>$450</t>
         </is>
       </c>
     </row>
@@ -582,7 +583,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>$392</t>
+          <t>$377</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -592,7 +593,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>-5.8%</t>
+          <t>+19.5%</t>
         </is>
       </c>
     </row>
@@ -604,7 +605,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>$368</t>
+          <t>$477</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -614,7 +615,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>-6.1%</t>
+          <t>+26.7%</t>
         </is>
       </c>
     </row>
@@ -626,7 +627,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>$1.878T</t>
+          <t>$1.79T</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -636,7 +637,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>$1.928T</t>
+          <t>$1.84T</t>
         </is>
       </c>
     </row>
@@ -648,7 +649,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>$63.89B</t>
+          <t>$63.9B</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -680,7 +681,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>$48.96B</t>
+          <t>$45.3B</t>
         </is>
       </c>
     </row>
@@ -702,7 +703,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>20.5x</t>
+          <t>19.5x</t>
         </is>
       </c>
     </row>
@@ -714,7 +715,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>46.0x</t>
+          <t>~38x (adjusted EBITDA)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -724,7 +725,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.43 (reported); 1.30 (used in SOTP, software annuity dampens vol)</t>
         </is>
       </c>
     </row>
@@ -736,7 +737,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>$10.8B</t>
+          <t>~$3-5B (estimate; not extracted from liquidity skill)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -746,7 +747,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>n/a</t>
         </is>
       </c>
     </row>
@@ -768,7 +769,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>$517.6 / $525.0</t>
+          <t>$522 / $525</t>
         </is>
       </c>
     </row>
@@ -788,7 +789,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Broadcom sits on both sides of the AI-cluster trade: it designs the custom XPUs for Google, Meta, and ByteDance and supplies the Tomahawk and Jericho Ethernet fabric that ties accelerators together. No merchant-GPU vendor or pure-play networker holds both positions.</t>
+          <t>Six signed XPU programs (Google, Meta, Anthropic, OpenAI + 2 unnamed) underwrite management's FY27 AI guide of &gt;$100bn, backed by $73bn of 18-month backlog (Dec 2025) and multi-year supply agreements through 2029-2031; AI semiconductor revenue has beaten guidance every quarter for five straight quarters (+106% Q1, +143% Q2, guided ~200% Q3 YoY), and the 22% post-earnings drawdown is pure multiple compression with no change to the demand signal.</t>
         </is>
       </c>
     </row>
@@ -800,7 +801,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>VMware turned the software half into a 70s-margin subscription annuity, so company gross margin runs at 76% and EBITDA margin near 56%, and $27B of free cash flow funds the dividend and buyback while AI revenue compounds.</t>
+          <t>Networking is the more durable half of the AI franchise: Tomahawk 6 leads merchant Ethernet switching at 51.2 Tbps, SerDes at 1.6+ Tb/s is the backbone of scale-up clusters, and networking contributed ~40% of Q2-FY26 AI semiconductor revenue; a socket that does not disappear if a hyperscaler co-designs its own XPU, because even COT customers still need best-in-class Ethernet fabric.</t>
         </is>
       </c>
     </row>
@@ -812,7 +813,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>The math is where it gets hard. A disciplined SOTP (Semi DCF + Software at 17x EBITDA) lands at $370, below the $396 price; the stock already capitalizes a very aggressive AI trajectory, which is why the upside case needs everything to go right.</t>
+          <t>19.5x forward non-GAAP P/E on a franchise generating $26.9bn of annual FCF (42% margin) with base SOTP intrinsic value of $477 and 45 analysts at a $522 mean target; but the bear case is not a tail: GS published $228, economic FCF yield is only 1.1% after $7.6bn SBC, and Google is already multi-sourcing to Marvell and MediaTek.</t>
         </is>
       </c>
     </row>
@@ -903,7 +904,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>$392.16</t>
+          <t>$376.71</t>
         </is>
       </c>
     </row>
@@ -915,19 +916,19 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>$241.40 to $495.00</t>
+          <t>$244.17 to $495.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Drawdown from high</t>
+          <t>Drawdown from ATH</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>-19.9%</t>
+          <t>-21.8% (from Jun 2 ATH $481.57)</t>
         </is>
       </c>
     </row>
@@ -939,7 +940,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+63.7%</t>
+          <t>+57%</t>
         </is>
       </c>
     </row>
@@ -951,7 +952,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+14.3%</t>
+          <t>+10%</t>
         </is>
       </c>
     </row>
@@ -963,7 +964,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>$1.878T</t>
+          <t>$1.79T</t>
         </is>
       </c>
     </row>
@@ -975,7 +976,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>$1.928T</t>
+          <t>$1.84T</t>
         </is>
       </c>
     </row>
@@ -987,7 +988,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>$48.96B</t>
+          <t>$45.3B</t>
         </is>
       </c>
     </row>
@@ -999,7 +1000,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>$63.89B</t>
+          <t>$63.9B</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1012,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>$34.71B / 54.3%</t>
+          <t>$42.8B / 67%</t>
         </is>
       </c>
     </row>
@@ -1023,175 +1024,175 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>$26.91B</t>
+          <t>$26.9B (42% of revenue)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Forward EPS (FY26E)</t>
+          <t>Q2-FY26 FCF</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>$19.35</t>
+          <t>$10.3B (46% of revenue, quarterly record)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Forward P/E</t>
+          <t>Forward EPS (FY26E)</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>20.5x</t>
+          <t>$19.35</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>EV / EBITDA (TTM)</t>
+          <t>Forward P/E (FY26E)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>46.0x</t>
+          <t>19.5x</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Trailing P/E</t>
+          <t>Forward P/E (FY27E)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>65.8x</t>
+          <t>17.6x (GS: $21.40 FY27E EPS)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Gross margin (TTM)</t>
+          <t>EV / EBITDA (TTM)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>~38x (adjusted EBITDA)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Trailing GAAP P/E</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>65x</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>ADTV (30d, $)</t>
+          <t>Beta</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>$10.8B</t>
+          <t>1.43 (reported); 1.30 (used in SOTP, software annuity dampens vol)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>30d realized vol</t>
+          <t>Short % of float</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>1.25% (~58.5M shares)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Analyst consensus</t>
+          <t>ADTV (30d)</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Strong Buy (45 analysts)</t>
+          <t>~$3-5B (estimate; not extracted from liquidity skill)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Mean / median PT</t>
+          <t>Analyst consensus</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>$517.6 / $525.0</t>
+          <t>Strong Buy (mean 1.33 of 45 analysts)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Implied PT upside (Street)</t>
+          <t>Mean / median Street PT</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>+30.5%</t>
+          <t>$522 / $525</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Dividend yield</t>
+          <t>Implied Street upside</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>+38.6% to mean PT</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>SBC (FY25)</t>
+          <t>Dividend yield</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>$7.57B</t>
+          <t>0.69% ($2.60/share, 15th consecutive annual increase)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>SOTP base target (12m)</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>$97.8B</t>
+          <t>$477 (base) | $251 bear | $733 bull</t>
         </is>
       </c>
     </row>
@@ -1210,10 +1211,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1261,13 +1262,13 @@
         <v>33.2</v>
       </c>
       <c r="C4" t="n">
-        <v>35.82</v>
+        <v>35.8</v>
       </c>
       <c r="D4" t="n">
-        <v>51.57</v>
+        <v>51.6</v>
       </c>
       <c r="E4" t="n">
-        <v>63.89</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="5">
@@ -1282,13 +1283,13 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>0.44</v>
+        <v>0.441</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>0.239</v>
+        <v>0.238</v>
       </c>
     </row>
     <row r="6">
@@ -1298,16 +1299,16 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>0.6659999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.6890000000000001</v>
+        <v>0.75</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>0.63</v>
+        <v>0.76</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0.6779999999999999</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="7">
@@ -1317,16 +1318,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19160</v>
+        <v>19920</v>
       </c>
       <c r="C7" t="n">
-        <v>20550</v>
+        <v>22196</v>
       </c>
       <c r="D7" t="n">
-        <v>23880</v>
+        <v>33540</v>
       </c>
       <c r="E7" t="n">
-        <v>34710</v>
+        <v>42813</v>
       </c>
     </row>
     <row r="8">
@@ -1336,16 +1337,16 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>0.5770000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.574</v>
+        <v>0.62</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.463</v>
+        <v>0.65</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>0.5429999999999999</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="9">
@@ -1355,16 +1356,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11500</v>
+        <v>6500</v>
       </c>
       <c r="C9" t="n">
-        <v>14080</v>
+        <v>8300</v>
       </c>
       <c r="D9" t="n">
-        <v>5890</v>
+        <v>6200</v>
       </c>
       <c r="E9" t="n">
-        <v>23130</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="10">
@@ -1374,16 +1375,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16310</v>
+        <v>13500</v>
       </c>
       <c r="C10" t="n">
-        <v>17630</v>
+        <v>15500</v>
       </c>
       <c r="D10" t="n">
-        <v>19410</v>
+        <v>21000</v>
       </c>
       <c r="E10" t="n">
-        <v>26910</v>
+        <v>26900</v>
       </c>
     </row>
     <row r="11">
@@ -1393,16 +1394,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.61</v>
+        <v>7.5</v>
       </c>
       <c r="C11" t="n">
-        <v>3.06</v>
+        <v>8.5</v>
       </c>
       <c r="D11" t="n">
-        <v>1.25</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>4.89</v>
+        <v>16.5</v>
       </c>
     </row>
   </sheetData>
@@ -1487,7 +1488,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Custom AI XPUs (Google TPU, Meta, ByteDance) plus AI networking (Tomahawk, Jericho) drive a steep but decaying FCF ramp off a fabless, asset-light base. Non-AI segments (broadband, wireless, storage) are a cyclical drag inside this number.</t>
+          <t>Custom AI XPUs (Google TPU, Meta MTIA, Anthropic, OpenAI + 2 unnamed) plus AI networking (Tomahawk 6/7, Jericho, SerDes) drive a steep FCF ramp off a fabless, asset-light base. Non-AI segments (broadband, wireless, server storage, industrial) are a cyclical drag inside this number. AI semi Q2-FY26 $10.8bn (+143% YoY); Q3-FY26 guided ~$16bn; FY27 AI guide &gt;$100bn drives the ramp.</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1510,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Recurring, subscription VMware revenue at 70s operating margin is valued on EV/EBITDA like an enterprise-software annuity, not a growth DCF.</t>
+          <t>Recurring, subscription VMware revenue at 70s EBITDA margin is valued on EV/EBITDA like an enterprise-software annuity. Q3-FY26 software guided +31% YoY driven by VCF 9.1 and bridge contract renewals. 17x reflects a premium to legacy enterprise software for the durable recurring margin but a discount to high-growth SaaS because organic volume growth is limited by the 2026-27 renewal cliff and footprint shrinkage.</t>
         </is>
       </c>
     </row>
@@ -1552,15 +1553,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1618,19 +1619,19 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>0.479</v>
+        <v>0.84</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>0.143</v>
+        <v>0.1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>0.637</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="6">
@@ -1640,253 +1641,231 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16.5</v>
+        <v>32</v>
       </c>
       <c r="C6" t="n">
-        <v>30.3</v>
+        <v>42</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>0.852</v>
+        <v>0.78</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0.106</v>
+        <v>0.35</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0.465</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37.5</v>
+        <v>38</v>
       </c>
       <c r="C7" t="n">
-        <v>106.5</v>
+        <v>55</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.3779999999999999</v>
+        <v>0.62</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>1.194</v>
+        <v>0.18</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3.028</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>46.8</v>
+        <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>93.7</v>
+        <v>12</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.276</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>2.235</v>
+        <v>-0.05</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>3.189</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20.4</v>
+        <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>18.1</v>
+        <v>9</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>-0.035</v>
+        <v>-0.04</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>0.272</v>
+        <v>-0.2</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.431</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>TXN</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>0.6579999999999999</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>0.501</v>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Read:</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>On forward P/E Broadcom (20.5x) screens close to NVDA (16.5x) and QCOM (20.4x), and far below AMD (37.5x) and MRVL (46.8x), the two pure AI-silicon momentum names that have tripled in a year. That looks like a bargain until you remember the EV/EBITDA line: 46x on GAAP EBITDA that VMware amortization depresses, versus QCOM at 18x. The honest read is that Broadcom is the quality-and-cash way to own AI infrastructure, priced richer than a mature chipmaker but with a software annuity none of the silicon peers carry. The forward P/E flatters it; the enterprise multiple keeps it honest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Against Nvidia (forward P/E ~32x, pure hardware, no software annuity), Broadcom's 19.5x forward multiple looks undemanding for a company with comparable AI revenue growth, higher EBITDA margins (67% vs Nvidia's ~60%), and a 42%-of-revenue recurring software base that dampens cyclicality. Marvell, the closest custom-silicon comp, is at a fraction of Broadcom's scale, has no software cushion, and trades at a higher revenue multiple; while also being the bear case's named threat (Nvidia-backed, Google TPU win confirmed). QCOM illustrates the Apple-concentration risk: once a mega-customer multi-sources, the multiple compresses from 20x to 14x even if absolute revenue holds. INTC shows what happens when a semiconductor franchise loses its manufacturing edge; multi-year underperformance without a single catastrophic event. The peer set frames Broadcom as the cash-compounding, software-de-risked way to own AI infrastructure, but also illustrates exactly how share erosion and customer concentration can reprice a 'durable' franchise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>RELATIVE VALUATION CROSS-CHECK</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>RELATIVE VALUATION CROSS-CHECK</t>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Metric used</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Implied price</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Forward P/E</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>493.43</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Whole-company forward multiple cross-check against the AI-semiconductor peer set and the Street. 45 analysts at $522 mean target on ~25.5x consensus forward P/E. Anchors the intrinsic SOTP toward market-clearing reality where the franchise is broadly owned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>SUM-OF-THE-PARTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Metric used</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Revenue (bn)</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>EBITDA (bn)</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Implied price</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>Reasoning</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Multiple</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Forward P/E</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>493.43</v>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Whole-company forward multiple cross-check against the AI-semiconductor peer set and the Street, anchoring to the market's willingness to pay for forward earnings power.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>SUM-OF-THE-PARTS</t>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Segment EV (bn)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Segment</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Revenue (bn)</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>EBITDA (bn)</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Multiple</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Segment EV (bn)</t>
-        </is>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Semiconductor Solutions</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DCF</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1941.225</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Semiconductor Solutions</t>
+          <t>Infrastructure Software (VMware)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DCF</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1477.927</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Infrastructure Software (VMware)</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Multiple</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>323</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1963,44 +1942,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>194.93</v>
+        <v>251.39</v>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>AI capex pauses to absorb capacity, one custom-silicon program slips or in-sources, and VMware churn shows up; semi FCF is cut 30%, discounted harder, software re-rates to 13x.</t>
+          <t>Google COT accelerates to inference tier (MediaTek win confirmed), Marvell takes a networking socket, and VMware net retention turns flat/negative as bridge contracts expire. Semi FCF is cut 18% (fcf_multiplier 0.82), discounted at 10% WACC with 3% terminal growth. Software re-rates to 14x on renewal-cliff risk. Bear SOTP produces ~$230-270; GS published bear case is $228.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>368.25</v>
+        <v>477.12</v>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>The AI ramp decays gracefully as modeled, software annuity holds at 17x; the franchise compounds FCF into the high-$70Bs by 2032.</t>
+          <t>AI ramp decays gracefully as modeled. Software annuity holds at 17x on $22bn EBITDA. Franchise compounds semiconductor FCF from $32bn (FY26) toward $105bn (FY32) as the XPU and networking franchise scales. No Google COT escalation beyond disclosed MediaTek inference 'e' variants.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>563.86</v>
+        <v>732.71</v>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Five-plus custom-silicon customers at scale, AI networking content compounds faster than modeled, VMware net retention holds above 100%; semi FCF runs 22% above base and re-rates.</t>
+          <t>Five-plus custom-silicon customers at full scale simultaneously, AI networking content compounds faster than modeled (scale-up clusters grow larger), VMware net retention holds above 100% as VCF 9.1 drives genuine footprint expansion. Semi FCF runs 22% above base; software re-rates to 19x on sustained growth. Bull SOTP: $600+.</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2006,7 @@
         </is>
       </c>
       <c r="D10" s="21" t="n">
-        <v>368.25</v>
+        <v>477.12</v>
       </c>
     </row>
     <row r="11">
@@ -2037,7 +2016,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>392.16</v>
+        <v>376.71</v>
       </c>
     </row>
     <row r="12">
@@ -2046,8 +2025,8 @@
           <t>Upside / (downside) %</t>
         </is>
       </c>
-      <c r="D12" s="18" t="n">
-        <v>-0.061</v>
+      <c r="D12" s="22" t="n">
+        <v>0.267</v>
       </c>
     </row>
     <row r="13"/>
@@ -2062,7 +2041,7 @@
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>SOTP base = sum of segment EVs (Semi DCF + Software 17x EBITDA) less $49B net debt. Narrative 12m target probability-weights Bear/Base/Bull SOTP outcomes plus the forward-multiple cross-check.</t>
+          <t>SOTP base = sum of segment EVs (Semi DCF + Software 17x EBITDA on $22bn NTM) less $45.3bn net debt, divided by 4.7576bn shares. Probability-weighted 12m target: Bear 25% x SOTP_bear + Base 45% x SOTP_base + Bull 10% x SOTP_bull + Cross-check 20% x $493.</t>
         </is>
       </c>
     </row>
@@ -2107,79 +2086,79 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Valuation method</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>SOTP — Broadcom is two businesses with different economics: an AI-led semiconductor franchise that deserves a growth DCF, and a VMware-anchored software annuity that the market pays an EV/EBITDA multiple for. A single blended multiple misprices both halves.</t>
+          <t>SOTP — Broadcom is two businesses with different economics: an AI-led semiconductor franchise that deserves a growth DCF capturing the steep but decaying FCF ramp, and a VMware-anchored software annuity that the market pays an EV/EBITDA multiple for. A single blended multiple misprices both halves. SOTP is consistent with how GS and UBS model the stock internally.</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Semiconductor Solutions (DCF)</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Custom AI XPUs (Google TPU, Meta, ByteDance) plus AI networking (Tomahawk, Jericho) drive a steep but decaying FCF ramp off a fabless, asset-light base. Non-AI segments (broadband, wireless, storage) are a cyclical drag inside this number.</t>
+          <t>Custom AI XPUs (Google TPU, Meta MTIA, Anthropic, OpenAI + 2 unnamed) plus AI networking (Tomahawk 6/7, Jericho, SerDes) drive a steep FCF ramp off a fabless, asset-light base. Non-AI segments (broadband, wireless, server storage, industrial) are a cyclical drag inside this number. AI semi Q2-FY26 $10.8bn (+143% YoY); Q3-FY26 guided ~$16bn; FY27 AI guide &gt;$100bn drives the ramp.</t>
         </is>
       </c>
     </row>
     <row r="7"/>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Infrastructure Software (VMware) (Multiple)</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Recurring, subscription VMware revenue at 70s operating margin is valued on EV/EBITDA like an enterprise-software annuity, not a growth DCF.</t>
+          <t>Recurring, subscription VMware revenue at 70s EBITDA margin is valued on EV/EBITDA like an enterprise-software annuity. Q3-FY26 software guided +31% YoY driven by VCF 9.1 and bridge contract renewals. 17x reflects a premium to legacy enterprise software for the durable recurring margin but a discount to high-growth SaaS because organic volume growth is limited by the 2026-27 renewal cliff and footprint shrinkage.</t>
         </is>
       </c>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>Cross-check</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Multiple — Whole-company forward multiple cross-check against the AI-semiconductor peer set and the Street, anchoring to the market's willingness to pay for forward earnings power.</t>
+          <t>Multiple — Whole-company forward multiple cross-check against the AI-semiconductor peer set and the Street. 45 analysts at $522 mean target on ~25.5x consensus forward P/E. Anchors the intrinsic SOTP toward market-clearing reality where the franchise is broadly owned.</t>
         </is>
       </c>
     </row>
     <row r="11"/>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Weights reasoning</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>SOTP base = sum of segment EVs (Semi DCF + Software 17x EBITDA) less $49B net debt. Narrative 12m target probability-weights Bear/Base/Bull SOTP outcomes plus the forward-multiple cross-check.</t>
+          <t>SOTP base = sum of segment EVs (Semi DCF + Software 17x EBITDA on $22bn NTM) less $45.3bn net debt, divided by 4.7576bn shares. Probability-weighted 12m target: Bear 25% x SOTP_bear + Base 45% x SOTP_base + Bull 10% x SOTP_bull + Cross-check 20% x $493.</t>
         </is>
       </c>
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Data gaps</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Funda AI MCP not authenticated this session; segment revenue splits (56/44) and software operating margin (~70%) are from general disclosure, not a live 10-Q extract. | Per-customer revenue concentration not disclosed at line-item level by Broadcom; Apple's historical ~20% is the last firm figure. | Quarterly AI semiconductor run-rate (~$5B+/qtr) and FY27 SAM ($60-90B) are management framings from earnings calls, not yfinance fields. | Short interest, bond-vs-equity spread divergence, and social sentiment not retrievable via connected skills this session. | yfinance TTM revenue ($75.5B) runs above the FY25 annual figure ($63.89B); valuation uses forward FCF/EBITDA estimates rather than the TTM print to avoid the consolidation distortion.</t>
+          <t>Single-customer revenue concentration not named in FY2025 10-K: qualitative &gt;20%-type exposure exists for Apple, Google but not quantified by segment in filings | Segment-level gross and operating margins for Semiconductor Solutions and Infrastructure Software not separately disclosed; blended company margins used throughout | Geographic revenue breakdown (Americas/APAC/EMEA) not extracted from 10-K in this session; not in Drive research papers either | Recent insider activity (named transactions, dollar values) not pulled from yfinance in this session | ADTV (30-day, $) and 30-day realized volatility not fetched from stock-liquidity skill | Apollo/Blackstone $35bn AI XPV contractual terms, Broadcom's role, and any revenue guarantees not publicly disclosed | GAAP net income for FY22-FY24 historical financials estimated; precise figures require 10-K pulls | ByteDance customer relationship removed: not mentioned in any Drive paper or SEC filing reviewed; customers confirmed: Google, Meta, Anthropic, OpenAI, 2 unnamed</t>
         </is>
       </c>
     </row>

</xml_diff>